<commit_message>
fix optimizer_pobo_sa.py, add similarity computation
</commit_message>
<xml_diff>
--- a/auto-configure/vdtuner/perf-predict-model/dataset_features.xlsx
+++ b/auto-configure/vdtuner/perf-predict-model/dataset_features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dzhdx\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{524B51E2-B1F6-4947-B5E4-7CF6604E505E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9607C99C-BEB0-4CBE-8AA1-0E5BB98D82D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{2B1B7960-0FA7-4219-8E33-0E691F8D4585}"/>
   </bookViews>
@@ -83,9 +83,6 @@
     <t>random-geo-radius-100-angular/random_geo_1m_no_filters</t>
   </si>
   <si>
-    <t>random_match_keyword</t>
-  </si>
-  <si>
     <t>random-geo-radius-2048-angular-no-filters</t>
   </si>
   <si>
@@ -104,6 +101,10 @@
   </si>
   <si>
     <t>gist-960-angular</t>
+  </si>
+  <si>
+    <t>random-match-keyword</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -489,6 +490,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B487134-60FE-49F3-B004-FA29A68043B4}">
   <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.1" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="30.3984375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
@@ -684,7 +688,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>100</v>
@@ -716,7 +720,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>2048</v>
@@ -748,7 +752,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>256</v>
@@ -780,7 +784,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <v>2048</v>
@@ -812,7 +816,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>2048</v>
@@ -844,7 +848,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <v>384</v>
@@ -876,7 +880,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B13">
         <v>960</v>

</xml_diff>